<commit_message>
feat(P4): Enterprise AI Governance & Technical Lifecycle
</commit_message>
<xml_diff>
--- a/04-ai-governance-and-technical-lifecycle/artifacts/A-11_Risk_Treatment_Plan.xlsx
+++ b/04-ai-governance-and-technical-lifecycle/artifacts/A-11_Risk_Treatment_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Career\Portfolio\Project4\Artifacts V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BD0D4FE-3E98-40A9-9CEA-6794117961BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{618794A8-6528-4FEB-9BBF-603C27D82E57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -71,9 +71,6 @@
     <t>Completed / Verified</t>
   </si>
   <si>
-    <t>Active in Production</t>
-  </si>
-  <si>
     <t>Accepted with Condition</t>
   </si>
   <si>
@@ -1222,6 +1219,9 @@
   <si>
     <t xml:space="preserve">
 R-11</t>
+  </si>
+  <si>
+    <t>Active - Scenario  Production</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1469,6 +1469,21 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1478,22 +1493,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1806,7 +1805,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1814,11 +1813,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:2" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
+    <row r="4" spans="1:2" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="28" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1865,26 +1864,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
-        <v>392</v>
-      </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
+      <c r="A1" s="35" t="s">
+        <v>391</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="B2" s="34"/>
+      <c r="C2" s="34"/>
+      <c r="D2" s="34"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="34"/>
     </row>
     <row r="4" spans="1:7" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
@@ -1897,21 +1896,21 @@
         <v>12</v>
       </c>
       <c r="D4" s="6" t="s">
+        <v>396</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" s="8">
         <v>18</v>
@@ -1926,15 +1925,15 @@
         <v>0</v>
       </c>
       <c r="F5" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>18</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="8">
         <v>1</v>
@@ -1949,15 +1948,15 @@
         <v>0</v>
       </c>
       <c r="F6" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" s="11" t="s">
         <v>21</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B7" s="8">
         <v>1</v>
@@ -1972,15 +1971,15 @@
         <v>1</v>
       </c>
       <c r="F7" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>24</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" s="8">
         <v>0</v>
@@ -1995,15 +1994,15 @@
         <v>0</v>
       </c>
       <c r="F8" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="11" t="s">
         <v>27</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" s="14">
         <v>20</v>
@@ -2018,20 +2017,20 @@
         <v>1</v>
       </c>
       <c r="F9" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="13" t="s">
-        <v>31</v>
-      </c>
     </row>
     <row r="15" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="30"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="29"/>
-      <c r="D15" s="29"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="29"/>
-      <c r="G15" s="29"/>
+      <c r="A15" s="35"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2059,99 +2058,99 @@
   <sheetData>
     <row r="1" spans="1:7" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="28" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
+      <c r="B4" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="C4" s="28" t="s">
         <v>34</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="D4" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="32" t="s">
+      <c r="E4" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="32" t="s">
+      <c r="F4" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="F4" s="32" t="s">
+      <c r="G4" s="28" t="s">
         <v>38</v>
-      </c>
-      <c r="G4" s="32" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -2183,120 +2182,120 @@
   <sheetData>
     <row r="1" spans="1:24" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" s="33" customFormat="1" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" s="29" customFormat="1" ht="28.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="G4" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="K4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="L4" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="M4" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="N4" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="N4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="O4" s="6" t="s">
+      <c r="P4" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q4" s="36"/>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="36"/>
-      <c r="V4" s="36"/>
-      <c r="W4" s="36"/>
-      <c r="X4" s="36"/>
+      <c r="Q4" s="31"/>
+      <c r="R4" s="31"/>
+      <c r="S4" s="31"/>
+      <c r="T4" s="31"/>
+      <c r="U4" s="31"/>
+      <c r="V4" s="31"/>
+      <c r="W4" s="31"/>
+      <c r="X4" s="31"/>
     </row>
     <row r="5" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="C5" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="D5" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F5" s="18" t="s">
+      <c r="G5" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="H5" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="H5" s="18" t="s">
+      <c r="I5" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="J5" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="K5" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="L5" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="L5" s="17" t="s">
+      <c r="M5" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="M5" s="18" t="s">
+      <c r="N5" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="N5" s="19" t="s">
+      <c r="O5" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="O5" s="18" t="s">
+      <c r="P5" s="18" t="s">
         <v>84</v>
-      </c>
-      <c r="P5" s="18" t="s">
-        <v>85</v>
       </c>
       <c r="Q5" s="15"/>
       <c r="R5" s="15"/>
@@ -2309,52 +2308,52 @@
     </row>
     <row r="6" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="18" t="s">
+      <c r="D6" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="F6" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="G6" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="H6" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="I6" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L6" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="M6" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="I6" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="J6" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="K6" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L6" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="M6" s="18" t="s">
+      <c r="N6" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O6" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="N6" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O6" s="18" t="s">
+      <c r="P6" s="18" t="s">
         <v>94</v>
-      </c>
-      <c r="P6" s="18" t="s">
-        <v>95</v>
       </c>
       <c r="Q6" s="15"/>
       <c r="R6" s="15"/>
@@ -2367,52 +2366,52 @@
     </row>
     <row r="7" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>97</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="G7" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="H7" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="I7" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="I7" s="17" t="s">
+      <c r="J7" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="J7" s="16" t="s">
+      <c r="K7" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="L7" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="M7" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="L7" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="M7" s="18" t="s">
+      <c r="N7" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O7" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="N7" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O7" s="18" t="s">
+      <c r="P7" s="18" t="s">
         <v>107</v>
-      </c>
-      <c r="P7" s="18" t="s">
-        <v>108</v>
       </c>
       <c r="Q7" s="15"/>
       <c r="R7" s="15"/>
@@ -2425,52 +2424,52 @@
     </row>
     <row r="8" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="B8" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="18" t="s">
+      <c r="D8" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="G8" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="H8" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="I8" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="J8" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="I8" s="17" t="s">
-        <v>103</v>
-      </c>
-      <c r="J8" s="16" t="s">
+      <c r="K8" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L8" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="M8" s="18" t="s">
         <v>116</v>
       </c>
-      <c r="K8" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L8" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="M8" s="18" t="s">
+      <c r="N8" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O8" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="N8" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O8" s="18" t="s">
+      <c r="P8" s="18" t="s">
         <v>118</v>
-      </c>
-      <c r="P8" s="18" t="s">
-        <v>119</v>
       </c>
       <c r="Q8" s="15"/>
       <c r="R8" s="15"/>
@@ -2483,52 +2482,52 @@
     </row>
     <row r="9" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="F9" s="18" t="s">
+      <c r="G9" s="18" t="s">
         <v>123</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="H9" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="I9" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="I9" s="17" t="s">
+      <c r="J9" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="K9" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L9" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="K9" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L9" s="17" t="s">
+      <c r="M9" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="M9" s="18" t="s">
+      <c r="N9" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="N9" s="19" t="s">
+      <c r="O9" s="18" t="s">
         <v>130</v>
       </c>
-      <c r="O9" s="18" t="s">
+      <c r="P9" s="18" t="s">
         <v>131</v>
-      </c>
-      <c r="P9" s="18" t="s">
-        <v>132</v>
       </c>
       <c r="Q9" s="15"/>
       <c r="R9" s="15"/>
@@ -2541,52 +2540,52 @@
     </row>
     <row r="10" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="E10" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F10" s="18" t="s">
+      <c r="G10" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="H10" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="H10" s="18" t="s">
+      <c r="I10" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="I10" s="17" t="s">
+      <c r="J10" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="K10" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L10" s="17" t="s">
         <v>140</v>
       </c>
-      <c r="K10" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L10" s="17" t="s">
+      <c r="M10" s="18" t="s">
         <v>141</v>
       </c>
-      <c r="M10" s="18" t="s">
+      <c r="N10" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O10" s="18" t="s">
         <v>142</v>
       </c>
-      <c r="N10" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O10" s="18" t="s">
+      <c r="P10" s="18" t="s">
         <v>143</v>
-      </c>
-      <c r="P10" s="18" t="s">
-        <v>144</v>
       </c>
       <c r="Q10" s="15"/>
       <c r="R10" s="15"/>
@@ -2599,52 +2598,52 @@
     </row>
     <row r="11" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="18" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11" s="18" t="s">
+      <c r="D11" s="18" t="s">
         <v>146</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="E11" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="E11" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="18" t="s">
+      <c r="G11" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="G11" s="18" t="s">
+      <c r="H11" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="I11" s="17" t="s">
         <v>150</v>
       </c>
-      <c r="I11" s="17" t="s">
+      <c r="J11" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="J11" s="16" t="s">
+      <c r="K11" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L11" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="M11" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="K11" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L11" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="M11" s="18" t="s">
+      <c r="N11" s="20" t="s">
         <v>153</v>
       </c>
-      <c r="N11" s="20" t="s">
+      <c r="O11" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="O11" s="18" t="s">
+      <c r="P11" s="18" t="s">
         <v>155</v>
-      </c>
-      <c r="P11" s="18" t="s">
-        <v>156</v>
       </c>
       <c r="Q11" s="15"/>
       <c r="R11" s="15"/>
@@ -2657,52 +2656,52 @@
     </row>
     <row r="12" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>157</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="18" t="s">
+      <c r="D12" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="E12" s="18" t="s">
         <v>159</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="F12" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="G12" s="18" t="s">
         <v>161</v>
       </c>
-      <c r="G12" s="18" t="s">
+      <c r="H12" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="18" t="s">
+      <c r="I12" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J12" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="I12" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J12" s="16" t="s">
+      <c r="K12" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L12" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="K12" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L12" s="17" t="s">
+      <c r="M12" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="M12" s="18" t="s">
+      <c r="N12" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O12" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="N12" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O12" s="18" t="s">
+      <c r="P12" s="18" t="s">
         <v>167</v>
-      </c>
-      <c r="P12" s="18" t="s">
-        <v>168</v>
       </c>
       <c r="Q12" s="15"/>
       <c r="R12" s="15"/>
@@ -2715,52 +2714,52 @@
     </row>
     <row r="13" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="18" t="s">
+      <c r="D13" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="E13" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="E13" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="18" t="s">
+      <c r="G13" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="G13" s="18" t="s">
+      <c r="H13" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="I13" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J13" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L13" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="I13" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J13" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="K13" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L13" s="17" t="s">
+      <c r="M13" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="M13" s="18" t="s">
+      <c r="N13" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O13" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="N13" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O13" s="18" t="s">
+      <c r="P13" s="18" t="s">
         <v>177</v>
-      </c>
-      <c r="P13" s="18" t="s">
-        <v>178</v>
       </c>
       <c r="Q13" s="15"/>
       <c r="R13" s="15"/>
@@ -2773,52 +2772,52 @@
     </row>
     <row r="14" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="18" t="s">
+      <c r="D14" s="18" t="s">
         <v>180</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="E14" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="F14" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="G14" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="G14" s="18" t="s">
+      <c r="H14" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="I14" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J14" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L14" s="17" t="s">
         <v>185</v>
       </c>
-      <c r="I14" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J14" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="K14" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L14" s="17" t="s">
+      <c r="M14" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="M14" s="18" t="s">
+      <c r="N14" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O14" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="N14" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O14" s="18" t="s">
+      <c r="P14" s="18" t="s">
         <v>188</v>
-      </c>
-      <c r="P14" s="18" t="s">
-        <v>189</v>
       </c>
       <c r="Q14" s="15"/>
       <c r="R14" s="15"/>
@@ -2831,52 +2830,52 @@
     </row>
     <row r="15" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="B15" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C15" s="18" t="s">
+      <c r="D15" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="E15" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="E15" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F15" s="18" t="s">
+      <c r="G15" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="G15" s="18" t="s">
+      <c r="H15" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="H15" s="18" t="s">
+      <c r="I15" s="17" t="s">
         <v>195</v>
       </c>
-      <c r="I15" s="17" t="s">
+      <c r="J15" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L15" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="M15" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="J15" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="K15" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L15" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="M15" s="18" t="s">
+      <c r="N15" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O15" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="N15" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O15" s="18" t="s">
+      <c r="P15" s="18" t="s">
         <v>198</v>
-      </c>
-      <c r="P15" s="18" t="s">
-        <v>199</v>
       </c>
       <c r="Q15" s="15"/>
       <c r="R15" s="15"/>
@@ -2889,52 +2888,52 @@
     </row>
     <row r="16" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="B16" s="17" t="s">
         <v>200</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="C16" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="D16" s="18" t="s">
         <v>202</v>
       </c>
-      <c r="D16" s="18" t="s">
+      <c r="E16" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="F16" s="18" t="s">
+      <c r="G16" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="G16" s="18" t="s">
+      <c r="H16" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="H16" s="18" t="s">
+      <c r="I16" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="I16" s="17" t="s">
+      <c r="J16" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="J16" s="16" t="s">
+      <c r="K16" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="K16" s="17" t="s">
+      <c r="L16" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="M16" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="L16" s="17" t="s">
-        <v>128</v>
-      </c>
-      <c r="M16" s="18" t="s">
+      <c r="N16" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="N16" s="21" t="s">
+      <c r="O16" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="O16" s="18" t="s">
+      <c r="P16" s="18" t="s">
         <v>213</v>
-      </c>
-      <c r="P16" s="18" t="s">
-        <v>214</v>
       </c>
       <c r="Q16" s="15"/>
       <c r="R16" s="15"/>
@@ -2947,52 +2946,52 @@
     </row>
     <row r="17" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="18" t="s">
         <v>215</v>
       </c>
-      <c r="B17" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C17" s="18" t="s">
+      <c r="D17" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="E17" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="E17" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="F17" s="18" t="s">
+      <c r="G17" s="18" t="s">
         <v>218</v>
       </c>
-      <c r="G17" s="18" t="s">
+      <c r="H17" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="H17" s="18" t="s">
+      <c r="I17" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="I17" s="17" t="s">
+      <c r="J17" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L17" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="M17" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="J17" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="K17" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L17" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="M17" s="18" t="s">
+      <c r="N17" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O17" s="18" t="s">
         <v>222</v>
       </c>
-      <c r="N17" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O17" s="18" t="s">
+      <c r="P17" s="18" t="s">
         <v>223</v>
-      </c>
-      <c r="P17" s="18" t="s">
-        <v>224</v>
       </c>
       <c r="Q17" s="15"/>
       <c r="R17" s="15"/>
@@ -3005,52 +3004,52 @@
     </row>
     <row r="18" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="16" t="s">
+        <v>224</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="E18" s="18" t="s">
-        <v>42</v>
-      </c>
-      <c r="F18" s="18" t="s">
+      <c r="G18" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="G18" s="18" t="s">
+      <c r="H18" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="H18" s="18" t="s">
+      <c r="I18" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J18" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="K18" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L18" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="M18" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="I18" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J18" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="K18" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L18" s="17" t="s">
-        <v>141</v>
-      </c>
-      <c r="M18" s="18" t="s">
+      <c r="N18" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O18" s="18" t="s">
         <v>231</v>
       </c>
-      <c r="N18" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O18" s="18" t="s">
+      <c r="P18" s="18" t="s">
         <v>232</v>
-      </c>
-      <c r="P18" s="18" t="s">
-        <v>233</v>
       </c>
       <c r="Q18" s="15"/>
       <c r="R18" s="15"/>
@@ -3063,52 +3062,52 @@
     </row>
     <row r="19" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="B19" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C19" s="18" t="s">
+      <c r="D19" s="18" t="s">
         <v>235</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="E19" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="F19" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="G19" s="18" t="s">
         <v>238</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="H19" s="18" t="s">
         <v>239</v>
       </c>
-      <c r="H19" s="18" t="s">
+      <c r="I19" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J19" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L19" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="M19" s="18" t="s">
         <v>240</v>
       </c>
-      <c r="I19" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J19" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="K19" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L19" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="M19" s="18" t="s">
+      <c r="N19" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O19" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="N19" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O19" s="18" t="s">
+      <c r="P19" s="18" t="s">
         <v>242</v>
-      </c>
-      <c r="P19" s="18" t="s">
-        <v>243</v>
       </c>
       <c r="Q19" s="15"/>
       <c r="R19" s="15"/>
@@ -3121,52 +3120,52 @@
     </row>
     <row r="20" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="18" t="s">
         <v>244</v>
       </c>
-      <c r="B20" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" s="18" t="s">
+      <c r="D20" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="F20" s="18" t="s">
         <v>246</v>
       </c>
-      <c r="E20" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="F20" s="18" t="s">
+      <c r="G20" s="18" t="s">
         <v>247</v>
       </c>
-      <c r="G20" s="18" t="s">
+      <c r="H20" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="H20" s="18" t="s">
+      <c r="I20" s="17" t="s">
         <v>249</v>
       </c>
-      <c r="I20" s="17" t="s">
+      <c r="J20" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="K20" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L20" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="M20" s="18" t="s">
         <v>250</v>
       </c>
-      <c r="J20" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="K20" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L20" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="M20" s="18" t="s">
+      <c r="N20" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="O20" s="18" t="s">
         <v>251</v>
       </c>
-      <c r="N20" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="O20" s="18" t="s">
+      <c r="P20" s="18" t="s">
         <v>252</v>
-      </c>
-      <c r="P20" s="18" t="s">
-        <v>253</v>
       </c>
       <c r="Q20" s="15"/>
       <c r="R20" s="15"/>
@@ -3179,52 +3178,52 @@
     </row>
     <row r="21" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
+        <v>253</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>254</v>
       </c>
-      <c r="B21" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C21" s="18" t="s">
+      <c r="D21" s="18" t="s">
         <v>255</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="F21" s="18" t="s">
         <v>256</v>
       </c>
-      <c r="E21" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="F21" s="18" t="s">
+      <c r="G21" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="G21" s="18" t="s">
+      <c r="H21" s="18" t="s">
         <v>258</v>
       </c>
-      <c r="H21" s="18" t="s">
+      <c r="I21" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J21" s="16" t="s">
         <v>259</v>
       </c>
-      <c r="I21" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J21" s="16" t="s">
+      <c r="K21" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L21" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="M21" s="18" t="s">
         <v>260</v>
       </c>
-      <c r="K21" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L21" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="M21" s="18" t="s">
+      <c r="N21" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O21" s="18" t="s">
         <v>261</v>
       </c>
-      <c r="N21" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O21" s="18" t="s">
+      <c r="P21" s="18" t="s">
         <v>262</v>
-      </c>
-      <c r="P21" s="18" t="s">
-        <v>263</v>
       </c>
       <c r="Q21" s="15"/>
       <c r="R21" s="15"/>
@@ -3237,52 +3236,52 @@
     </row>
     <row r="22" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
+        <v>263</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="18" t="s">
         <v>264</v>
       </c>
-      <c r="B22" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C22" s="18" t="s">
+      <c r="D22" s="18" t="s">
         <v>265</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>266</v>
       </c>
-      <c r="E22" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="F22" s="18" t="s">
+      <c r="G22" s="18" t="s">
         <v>267</v>
       </c>
-      <c r="G22" s="18" t="s">
+      <c r="H22" s="18" t="s">
         <v>268</v>
       </c>
-      <c r="H22" s="18" t="s">
+      <c r="I22" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J22" s="16" t="s">
         <v>269</v>
       </c>
-      <c r="I22" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J22" s="16" t="s">
+      <c r="K22" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L22" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="M22" s="18" t="s">
         <v>270</v>
       </c>
-      <c r="K22" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="L22" s="17" t="s">
-        <v>165</v>
-      </c>
-      <c r="M22" s="18" t="s">
+      <c r="N22" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O22" s="18" t="s">
         <v>271</v>
       </c>
-      <c r="N22" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O22" s="18" t="s">
+      <c r="P22" s="18" t="s">
         <v>272</v>
-      </c>
-      <c r="P22" s="18" t="s">
-        <v>273</v>
       </c>
       <c r="Q22" s="15"/>
       <c r="R22" s="15"/>
@@ -3295,52 +3294,52 @@
     </row>
     <row r="23" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
+        <v>273</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="18" t="s">
         <v>274</v>
       </c>
-      <c r="B23" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" s="18" t="s">
+      <c r="D23" s="18" t="s">
         <v>275</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>276</v>
       </c>
-      <c r="E23" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="F23" s="18" t="s">
+      <c r="G23" s="18" t="s">
         <v>277</v>
       </c>
-      <c r="G23" s="18" t="s">
+      <c r="H23" s="18" t="s">
         <v>278</v>
       </c>
-      <c r="H23" s="18" t="s">
+      <c r="I23" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J23" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L23" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="M23" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="I23" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J23" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="K23" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L23" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="M23" s="18" t="s">
+      <c r="N23" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O23" s="18" t="s">
         <v>280</v>
       </c>
-      <c r="N23" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O23" s="18" t="s">
+      <c r="P23" s="18" t="s">
         <v>281</v>
-      </c>
-      <c r="P23" s="18" t="s">
-        <v>282</v>
       </c>
       <c r="Q23" s="15"/>
       <c r="R23" s="15"/>
@@ -3353,52 +3352,52 @@
     </row>
     <row r="24" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
+        <v>282</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="18" t="s">
         <v>283</v>
       </c>
-      <c r="B24" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="C24" s="18" t="s">
+      <c r="D24" s="18" t="s">
         <v>284</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
         <v>285</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="F24" s="18" t="s">
         <v>286</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="G24" s="18" t="s">
         <v>287</v>
       </c>
-      <c r="G24" s="18" t="s">
+      <c r="H24" s="18" t="s">
         <v>288</v>
       </c>
-      <c r="H24" s="18" t="s">
+      <c r="I24" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J24" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="K24" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="L24" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="M24" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="I24" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="J24" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="K24" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="L24" s="17" t="s">
-        <v>175</v>
-      </c>
-      <c r="M24" s="18" t="s">
+      <c r="N24" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="O24" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="N24" s="20" t="s">
-        <v>154</v>
-      </c>
-      <c r="O24" s="18" t="s">
+      <c r="P24" s="18" t="s">
         <v>291</v>
-      </c>
-      <c r="P24" s="18" t="s">
-        <v>292</v>
       </c>
       <c r="Q24" s="15"/>
       <c r="R24" s="15"/>
@@ -3436,24 +3435,24 @@
       <c r="X25" s="15"/>
     </row>
     <row r="26" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A26" s="31" t="s">
-        <v>293</v>
-      </c>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="29"/>
-      <c r="L26" s="29"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="29"/>
-      <c r="O26" s="29"/>
-      <c r="P26" s="29"/>
+      <c r="A26" s="36" t="s">
+        <v>292</v>
+      </c>
+      <c r="B26" s="34"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="34"/>
+      <c r="J26" s="34"/>
+      <c r="K26" s="34"/>
+      <c r="L26" s="34"/>
+      <c r="M26" s="34"/>
+      <c r="N26" s="34"/>
+      <c r="O26" s="34"/>
+      <c r="P26" s="34"/>
       <c r="Q26" s="15"/>
       <c r="R26" s="15"/>
       <c r="S26" s="15"/>
@@ -3464,22 +3463,22 @@
       <c r="X26" s="15"/>
     </row>
     <row r="27" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A27" s="29"/>
-      <c r="B27" s="29"/>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="29"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="29"/>
-      <c r="L27" s="29"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="29"/>
-      <c r="O27" s="29"/>
-      <c r="P27" s="29"/>
+      <c r="A27" s="34"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="34"/>
+      <c r="J27" s="34"/>
+      <c r="K27" s="34"/>
+      <c r="L27" s="34"/>
+      <c r="M27" s="34"/>
+      <c r="N27" s="34"/>
+      <c r="O27" s="34"/>
+      <c r="P27" s="34"/>
       <c r="Q27" s="15"/>
       <c r="R27" s="15"/>
       <c r="S27" s="15"/>
@@ -4056,118 +4055,118 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" s="33" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="C4" s="6" t="s">
+    </row>
+    <row r="5" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="32" t="s">
+        <v>395</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>296</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
-        <v>396</v>
-      </c>
-      <c r="B5" s="18" t="s">
+      <c r="C5" s="18" t="s">
         <v>297</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>298</v>
       </c>
       <c r="D5" s="15"/>
     </row>
     <row r="6" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B6" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>299</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>300</v>
       </c>
       <c r="D6" s="15"/>
     </row>
     <row r="7" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B7" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="C7" s="18" t="s">
         <v>301</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>302</v>
       </c>
       <c r="D7" s="15"/>
     </row>
     <row r="8" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B8" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>303</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>304</v>
       </c>
       <c r="D8" s="15"/>
     </row>
     <row r="9" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B9" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="C9" s="18" t="s">
         <v>305</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>306</v>
       </c>
       <c r="D9" s="15"/>
     </row>
     <row r="10" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B10" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="C10" s="18" t="s">
         <v>307</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>308</v>
       </c>
       <c r="D10" s="15"/>
     </row>
     <row r="11" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B11" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="C11" s="18" t="s">
         <v>309</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>310</v>
       </c>
       <c r="D11" s="15"/>
     </row>
     <row r="12" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>311</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>312</v>
       </c>
       <c r="D12" s="15"/>
     </row>
@@ -4229,514 +4228,514 @@
   <sheetData>
     <row r="1" spans="1:8" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A4" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="30" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" s="35" customFormat="1" ht="26.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="34" t="s">
-        <v>43</v>
-      </c>
-      <c r="B4" s="34" t="s">
+      <c r="C4" s="30" t="s">
         <v>314</v>
       </c>
-      <c r="C4" s="34" t="s">
+      <c r="D4" s="30" t="s">
         <v>315</v>
       </c>
-      <c r="D4" s="34" t="s">
+      <c r="E4" s="30" t="s">
         <v>316</v>
       </c>
-      <c r="E4" s="34" t="s">
+      <c r="F4" s="30" t="s">
         <v>317</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="G4" s="30" t="s">
         <v>318</v>
-      </c>
-      <c r="G4" s="34" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B5" s="23" t="s">
+        <v>319</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>320</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="D5" s="24" t="s">
         <v>321</v>
       </c>
-      <c r="D5" s="24" t="s">
+      <c r="E5" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="23" t="s">
         <v>322</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" s="23" t="s">
-        <v>323</v>
       </c>
       <c r="H5" s="15"/>
     </row>
     <row r="6" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C6" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="D6" s="24" t="s">
         <v>324</v>
       </c>
-      <c r="D6" s="24" t="s">
-        <v>325</v>
-      </c>
       <c r="E6" s="23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H6" s="15"/>
     </row>
     <row r="7" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B7" s="23" t="s">
+        <v>325</v>
+      </c>
+      <c r="C7" s="24" t="s">
         <v>326</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="D7" s="24" t="s">
         <v>327</v>
       </c>
-      <c r="D7" s="24" t="s">
-        <v>328</v>
-      </c>
       <c r="E7" s="23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H7" s="15"/>
     </row>
     <row r="8" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C8" s="24" t="s">
+        <v>328</v>
+      </c>
+      <c r="D8" s="24" t="s">
         <v>329</v>
       </c>
-      <c r="D8" s="24" t="s">
-        <v>330</v>
-      </c>
       <c r="E8" s="23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H8" s="15"/>
     </row>
     <row r="9" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C9" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="D9" s="24" t="s">
         <v>331</v>
       </c>
-      <c r="D9" s="24" t="s">
-        <v>332</v>
-      </c>
       <c r="E9" s="23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H9" s="15"/>
     </row>
     <row r="10" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B10" s="23" t="s">
+        <v>332</v>
+      </c>
+      <c r="C10" s="24" t="s">
         <v>333</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="D10" s="24" t="s">
         <v>334</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="E10" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="23" t="s">
         <v>335</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>139</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>336</v>
       </c>
       <c r="H10" s="15"/>
     </row>
     <row r="11" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B11" s="26" t="s">
+        <v>336</v>
+      </c>
+      <c r="C11" s="27" t="s">
         <v>337</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="D11" s="27" t="s">
         <v>338</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="E11" s="26" t="s">
         <v>339</v>
       </c>
-      <c r="E11" s="26" t="s">
-        <v>340</v>
-      </c>
       <c r="F11" s="27" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H11" s="15"/>
     </row>
     <row r="12" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B12" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="D12" s="18" t="s">
         <v>342</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="E12" s="17" t="s">
         <v>343</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="F12" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="F12" s="18" t="s">
-        <v>345</v>
-      </c>
       <c r="G12" s="17" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H12" s="15"/>
     </row>
     <row r="13" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B13" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="C13" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="D13" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="E13" s="17" t="s">
         <v>348</v>
       </c>
-      <c r="E13" s="17" t="s">
-        <v>349</v>
-      </c>
       <c r="F13" s="18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H13" s="15"/>
     </row>
     <row r="14" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B14" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>350</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="D14" s="18" t="s">
         <v>351</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="E14" s="17" t="s">
         <v>352</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="F14" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="G14" s="17" t="s">
         <v>353</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>182</v>
-      </c>
-      <c r="G14" s="17" t="s">
-        <v>354</v>
       </c>
       <c r="H14" s="15"/>
     </row>
     <row r="15" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C15" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="D15" s="18" t="s">
         <v>355</v>
       </c>
-      <c r="D15" s="18" t="s">
-        <v>356</v>
-      </c>
       <c r="E15" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H15" s="15"/>
     </row>
     <row r="16" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B16" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="C16" s="18" t="s">
         <v>357</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="D16" s="18" t="s">
         <v>358</v>
       </c>
-      <c r="D16" s="18" t="s">
-        <v>359</v>
-      </c>
       <c r="E16" s="17" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H16" s="15"/>
     </row>
     <row r="17" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="16" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C17" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="D17" s="18" t="s">
         <v>360</v>
       </c>
-      <c r="D17" s="18" t="s">
+      <c r="E17" s="17" t="s">
         <v>361</v>
       </c>
-      <c r="E17" s="17" t="s">
-        <v>362</v>
-      </c>
       <c r="F17" s="18" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H17" s="15"/>
     </row>
     <row r="18" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="16" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B18" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="C18" s="18" t="s">
         <v>363</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="D18" s="18" t="s">
         <v>364</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="17" t="s">
         <v>365</v>
       </c>
-      <c r="E18" s="17" t="s">
-        <v>366</v>
-      </c>
       <c r="F18" s="18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H18" s="15"/>
     </row>
     <row r="19" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B19" s="17" t="s">
+        <v>366</v>
+      </c>
+      <c r="C19" s="18" t="s">
         <v>367</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="D19" s="18" t="s">
         <v>368</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="E19" s="17" t="s">
         <v>369</v>
       </c>
-      <c r="E19" s="17" t="s">
-        <v>370</v>
-      </c>
       <c r="F19" s="18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H19" s="15"/>
     </row>
     <row r="20" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="16" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C20" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="D20" s="18" t="s">
         <v>371</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="G20" s="17" t="s">
         <v>372</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>250</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>373</v>
       </c>
       <c r="H20" s="15"/>
     </row>
     <row r="21" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="16" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B21" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>374</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="D21" s="18" t="s">
         <v>375</v>
       </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="17" t="s">
         <v>376</v>
       </c>
-      <c r="E21" s="17" t="s">
-        <v>377</v>
-      </c>
       <c r="F21" s="18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H21" s="15"/>
     </row>
     <row r="22" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="16" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B22" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="C22" s="18" t="s">
         <v>378</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="D22" s="18" t="s">
         <v>379</v>
       </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="17" t="s">
         <v>380</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="F22" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="G22" s="17" t="s">
         <v>381</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>237</v>
-      </c>
-      <c r="G22" s="17" t="s">
-        <v>382</v>
       </c>
       <c r="H22" s="15"/>
     </row>
     <row r="23" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="16" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C23" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>383</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="17" t="s">
         <v>384</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="F23" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23" s="17" t="s">
         <v>385</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>99</v>
-      </c>
-      <c r="G23" s="17" t="s">
-        <v>386</v>
       </c>
       <c r="H23" s="15"/>
     </row>
     <row r="24" spans="1:8" ht="43.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="16" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B24" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="C24" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="D24" s="18" t="s">
         <v>388</v>
       </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="17" t="s">
         <v>389</v>
       </c>
-      <c r="E24" s="17" t="s">
-        <v>390</v>
-      </c>
       <c r="F24" s="18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="H24" s="15"/>
     </row>

</xml_diff>